<commit_message>
Analisi Finanziarie: Net Worth come il foglio, entrate come il foglio, cancellazione vera, temi, layout a tutta larghezza (in corso)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EU8iXu877ZDR8ixrLFK5MP
</commit_message>
<xml_diff>
--- a/finanza-personale/test/fixtures/file-completo-esempio.xlsx
+++ b/finanza-personale/test/fixtures/file-completo-esempio.xlsx
@@ -4672,7 +4672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4787,7 +4787,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Contanti</t>
+          <t>Trade Republic</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4796,393 +4796,393 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="D4" t="n">
-        <v>310</v>
+        <v>625</v>
       </c>
       <c r="E4" t="n">
-        <v>320</v>
+        <v>650</v>
       </c>
       <c r="F4" t="n">
-        <v>330</v>
+        <v>675</v>
       </c>
       <c r="G4" t="n">
-        <v>500000</v>
+        <v>700</v>
       </c>
       <c r="H4" t="n">
-        <v>350</v>
+        <v>725</v>
       </c>
       <c r="I4" t="n">
-        <v>360</v>
+        <v>750</v>
       </c>
       <c r="J4" t="n">
-        <v>370</v>
+        <v>775</v>
       </c>
       <c r="K4" t="n">
-        <v>380</v>
+        <v>800</v>
       </c>
       <c r="L4" t="n">
-        <v>390</v>
+        <v>825</v>
       </c>
       <c r="M4" t="n">
-        <v>400</v>
+        <v>850</v>
       </c>
       <c r="N4" t="n">
-        <v>410</v>
+        <v>875</v>
       </c>
       <c r="O4" t="n">
-        <v>420</v>
+        <v>900</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Conto USD</t>
+          <t>Scalable Capital</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dollari</t>
+          <t>Euro</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="D5" t="n">
-        <v>1200</v>
+        <v>2006.5</v>
       </c>
       <c r="E5" t="n">
-        <v>1200</v>
+        <v>2013</v>
       </c>
       <c r="F5" t="n">
-        <v>1200</v>
+        <v>2019.5</v>
       </c>
       <c r="G5" t="n">
-        <v>1200</v>
+        <v>2026</v>
       </c>
       <c r="H5" t="n">
-        <v>1200</v>
+        <v>2032.5</v>
       </c>
       <c r="I5" t="n">
-        <v>1200</v>
+        <v>2039</v>
       </c>
       <c r="J5" t="n">
-        <v>1200</v>
+        <v>2045.5</v>
       </c>
       <c r="K5" t="n">
-        <v>1200</v>
+        <v>2052</v>
       </c>
       <c r="L5" t="n">
-        <v>1200</v>
+        <v>2058.5</v>
       </c>
       <c r="M5" t="n">
-        <v>1200</v>
+        <v>2065</v>
       </c>
       <c r="N5" t="n">
-        <v>1200</v>
+        <v>2071.5</v>
       </c>
       <c r="O5" t="n">
-        <v>1200</v>
+        <v>2078</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Contanti</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Euro</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9500</v>
+        <v>300</v>
       </c>
       <c r="D6" t="n">
-        <v>9960</v>
+        <v>310</v>
       </c>
       <c r="E6" t="n">
-        <v>10420</v>
+        <v>320</v>
       </c>
       <c r="F6" t="n">
-        <v>10880</v>
+        <v>330</v>
       </c>
       <c r="G6" t="n">
-        <v>511000</v>
+        <v>500000</v>
       </c>
       <c r="H6" t="n">
-        <v>11800</v>
+        <v>350</v>
       </c>
       <c r="I6" t="n">
-        <v>12260</v>
+        <v>360</v>
       </c>
       <c r="J6" t="n">
-        <v>12720</v>
+        <v>370</v>
       </c>
       <c r="K6" t="n">
-        <v>13180</v>
+        <v>380</v>
       </c>
       <c r="L6" t="n">
-        <v>13640</v>
+        <v>390</v>
       </c>
       <c r="M6" t="n">
-        <v>14100</v>
+        <v>400</v>
       </c>
       <c r="N6" t="n">
-        <v>14560</v>
+        <v>410</v>
       </c>
       <c r="O6" t="n">
-        <v>15020</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gain/Loss</t>
-        </is>
+          <t>Conto USD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dollari</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1200</v>
       </c>
       <c r="D7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="E7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="F7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="G7" t="n">
-        <v>500120</v>
+        <v>1200</v>
       </c>
       <c r="H7" t="n">
-        <v>-499200</v>
+        <v>1200</v>
       </c>
       <c r="I7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="J7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="K7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="L7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="M7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="N7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
       <c r="O7" t="n">
-        <v>460</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>12100</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0484</v>
+        <v>12591.5</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0462</v>
+        <v>13083</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0441</v>
+        <v>13574.5</v>
       </c>
       <c r="G8" t="n">
-        <v>45.9669</v>
+        <v>513726</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.9769</v>
+        <v>14557.5</v>
       </c>
       <c r="I8" t="n">
-        <v>0.039</v>
+        <v>15049</v>
       </c>
       <c r="J8" t="n">
-        <v>0.0375</v>
+        <v>15540.5</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0362</v>
+        <v>16032</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0349</v>
+        <v>16523.5</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0337</v>
+        <v>17015</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0326</v>
+        <v>17506.5</v>
       </c>
       <c r="O8" t="n">
-        <v>0.0316</v>
-      </c>
-    </row>
-    <row r="9"/>
+        <v>17998</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gain/Loss</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>500151.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-499168.5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="L9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>491.5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>491.5</v>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ETF</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ETF</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>3500</v>
-      </c>
-      <c r="D11" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E11" t="n">
-        <v>4100</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4400</v>
-      </c>
-      <c r="G11" t="n">
-        <v>4700</v>
-      </c>
-      <c r="H11" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I11" t="n">
-        <v>5300</v>
-      </c>
-      <c r="J11" t="n">
-        <v>5600</v>
-      </c>
-      <c r="K11" t="n">
-        <v>5900</v>
-      </c>
-      <c r="L11" t="n">
-        <v>6200</v>
-      </c>
-      <c r="M11" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N11" t="n">
-        <v>6800</v>
-      </c>
-      <c r="O11" t="n">
-        <v>7100</v>
-      </c>
-    </row>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.039</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0376</v>
+      </c>
+      <c r="G10" t="n">
+        <v>36.8449</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.9717</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0338</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.0327</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.0307</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.0297</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.0289</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.0281</v>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Emerging Markets</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
           <t>ETF</t>
         </is>
-      </c>
-      <c r="C12" t="n">
-        <v>1300</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1700</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1900</v>
-      </c>
-      <c r="G12" t="n">
-        <v>2100</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2300</v>
-      </c>
-      <c r="I12" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2700</v>
-      </c>
-      <c r="K12" t="n">
-        <v>2900</v>
-      </c>
-      <c r="L12" t="n">
-        <v>3100</v>
-      </c>
-      <c r="M12" t="n">
-        <v>3300</v>
-      </c>
-      <c r="N12" t="n">
-        <v>3500</v>
-      </c>
-      <c r="O12" t="n">
-        <v>3700</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ETC</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1000</v>
+        <v>3500</v>
       </c>
       <c r="D13" t="n">
-        <v>1120</v>
+        <v>3800</v>
       </c>
       <c r="E13" t="n">
-        <v>1240</v>
+        <v>4100</v>
       </c>
       <c r="F13" t="n">
-        <v>1360</v>
+        <v>4400</v>
       </c>
       <c r="G13" t="n">
-        <v>1480</v>
+        <v>4700</v>
       </c>
       <c r="H13" t="n">
-        <v>1600</v>
+        <v>5000</v>
       </c>
       <c r="I13" t="n">
-        <v>1720</v>
+        <v>5300</v>
       </c>
       <c r="J13" t="n">
-        <v>1840</v>
+        <v>5600</v>
       </c>
       <c r="K13" t="n">
-        <v>1960</v>
+        <v>5900</v>
       </c>
       <c r="L13" t="n">
-        <v>2080</v>
+        <v>6200</v>
       </c>
       <c r="M13" t="n">
-        <v>2200</v>
+        <v>6500</v>
       </c>
       <c r="N13" t="n">
-        <v>2320</v>
+        <v>6800</v>
       </c>
       <c r="O13" t="n">
-        <v>2440</v>
+        <v>7100</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Xeon</t>
+          <t>Emerging Markets</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5191,871 +5191,973 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>1700</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1900</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>2100</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>2300</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>2900</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>3100</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>3300</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ETC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>5800</v>
+        <v>1000</v>
       </c>
       <c r="D15" t="n">
-        <v>6420</v>
+        <v>1120</v>
       </c>
       <c r="E15" t="n">
-        <v>7040</v>
+        <v>1240</v>
       </c>
       <c r="F15" t="n">
-        <v>7660</v>
+        <v>1360</v>
       </c>
       <c r="G15" t="n">
-        <v>8280</v>
+        <v>1480</v>
       </c>
       <c r="H15" t="n">
-        <v>8900</v>
+        <v>1600</v>
       </c>
       <c r="I15" t="n">
-        <v>9520</v>
+        <v>1720</v>
       </c>
       <c r="J15" t="n">
-        <v>10140</v>
+        <v>1840</v>
       </c>
       <c r="K15" t="n">
-        <v>10760</v>
+        <v>1960</v>
       </c>
       <c r="L15" t="n">
-        <v>11380</v>
+        <v>2080</v>
       </c>
       <c r="M15" t="n">
-        <v>12000</v>
+        <v>2200</v>
       </c>
       <c r="N15" t="n">
-        <v>12620</v>
+        <v>2320</v>
       </c>
       <c r="O15" t="n">
-        <v>13240</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Gain/Loss</t>
-        </is>
+          <t>Xeon</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
-        <v>620</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5800</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1069</v>
+        <v>6420</v>
       </c>
       <c r="E17" t="n">
-        <v>0.09660000000000001</v>
+        <v>7040</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0881</v>
+        <v>7660</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0809</v>
+        <v>8280</v>
       </c>
       <c r="H17" t="n">
-        <v>0.07489999999999999</v>
+        <v>8900</v>
       </c>
       <c r="I17" t="n">
-        <v>0.0697</v>
+        <v>9520</v>
       </c>
       <c r="J17" t="n">
-        <v>0.06510000000000001</v>
+        <v>10140</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0611</v>
+        <v>10760</v>
       </c>
       <c r="L17" t="n">
-        <v>0.0576</v>
+        <v>11380</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0545</v>
+        <v>12000</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0517</v>
+        <v>12620</v>
       </c>
       <c r="O17" t="n">
-        <v>0.0491</v>
-      </c>
-    </row>
-    <row r="18"/>
+        <v>13240</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Gain/Loss</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>620</v>
+      </c>
+      <c r="E18" t="n">
+        <v>620</v>
+      </c>
+      <c r="F18" t="n">
+        <v>620</v>
+      </c>
+      <c r="G18" t="n">
+        <v>620</v>
+      </c>
+      <c r="H18" t="n">
+        <v>620</v>
+      </c>
+      <c r="I18" t="n">
+        <v>620</v>
+      </c>
+      <c r="J18" t="n">
+        <v>620</v>
+      </c>
+      <c r="K18" t="n">
+        <v>620</v>
+      </c>
+      <c r="L18" t="n">
+        <v>620</v>
+      </c>
+      <c r="M18" t="n">
+        <v>620</v>
+      </c>
+      <c r="N18" t="n">
+        <v>620</v>
+      </c>
+      <c r="O18" t="n">
+        <v>620</v>
+      </c>
+    </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stock</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Rocket Lab</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Azione</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
-        <v>50</v>
-      </c>
-      <c r="E20" t="n">
-        <v>100</v>
-      </c>
-      <c r="F20" t="n">
-        <v>150</v>
-      </c>
-      <c r="G20" t="n">
-        <v>200</v>
-      </c>
-      <c r="H20" t="n">
-        <v>250</v>
-      </c>
-      <c r="I20" t="n">
-        <v>300</v>
-      </c>
-      <c r="J20" t="n">
-        <v>350</v>
-      </c>
-      <c r="K20" t="n">
-        <v>400</v>
-      </c>
-      <c r="L20" t="n">
-        <v>450</v>
-      </c>
-      <c r="M20" t="n">
-        <v>500</v>
-      </c>
-      <c r="N20" t="n">
-        <v>550</v>
-      </c>
-      <c r="O20" t="n">
-        <v>600</v>
-      </c>
-    </row>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.1069</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.09660000000000001</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0881</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0809</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.07489999999999999</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.0697</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.06510000000000001</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.0611</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.0576</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.0545</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.0517</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.0491</v>
+      </c>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>50</v>
-      </c>
-      <c r="E21" t="n">
-        <v>100</v>
-      </c>
-      <c r="F21" t="n">
-        <v>150</v>
-      </c>
-      <c r="G21" t="n">
-        <v>200</v>
-      </c>
-      <c r="H21" t="n">
-        <v>250</v>
-      </c>
-      <c r="I21" t="n">
-        <v>300</v>
-      </c>
-      <c r="J21" t="n">
-        <v>350</v>
-      </c>
-      <c r="K21" t="n">
-        <v>400</v>
-      </c>
-      <c r="L21" t="n">
-        <v>450</v>
-      </c>
-      <c r="M21" t="n">
-        <v>500</v>
-      </c>
-      <c r="N21" t="n">
-        <v>550</v>
-      </c>
-      <c r="O21" t="n">
-        <v>600</v>
+          <t>Stock</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Gain/Loss</t>
-        </is>
+          <t>Rocket Lab</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Azione</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>50</v>
       </c>
       <c r="E22" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F22" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="G22" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="H22" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="I22" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="J22" t="n">
-        <v>50</v>
+        <v>350</v>
       </c>
       <c r="K22" t="n">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="L22" t="n">
-        <v>50</v>
+        <v>450</v>
       </c>
       <c r="M22" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="N22" t="n">
-        <v>50</v>
+        <v>550</v>
       </c>
       <c r="O22" t="n">
-        <v>50</v>
+        <v>600</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>50</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F23" t="n">
-        <v>0.5</v>
+        <v>150</v>
       </c>
       <c r="G23" t="n">
-        <v>0.3333</v>
+        <v>200</v>
       </c>
       <c r="H23" t="n">
-        <v>0.25</v>
+        <v>250</v>
       </c>
       <c r="I23" t="n">
-        <v>0.2</v>
+        <v>300</v>
       </c>
       <c r="J23" t="n">
-        <v>0.1667</v>
+        <v>350</v>
       </c>
       <c r="K23" t="n">
-        <v>0.1429</v>
+        <v>400</v>
       </c>
       <c r="L23" t="n">
-        <v>0.125</v>
+        <v>450</v>
       </c>
       <c r="M23" t="n">
-        <v>0.1111</v>
+        <v>500</v>
       </c>
       <c r="N23" t="n">
-        <v>0.1</v>
+        <v>550</v>
       </c>
       <c r="O23" t="n">
-        <v>0.09089999999999999</v>
-      </c>
-    </row>
-    <row r="24"/>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Gain/Loss</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>50</v>
+      </c>
+      <c r="E24" t="n">
+        <v>50</v>
+      </c>
+      <c r="F24" t="n">
+        <v>50</v>
+      </c>
+      <c r="G24" t="n">
+        <v>50</v>
+      </c>
+      <c r="H24" t="n">
+        <v>50</v>
+      </c>
+      <c r="I24" t="n">
+        <v>50</v>
+      </c>
+      <c r="J24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K24" t="n">
+        <v>50</v>
+      </c>
+      <c r="L24" t="n">
+        <v>50</v>
+      </c>
+      <c r="M24" t="n">
+        <v>50</v>
+      </c>
+      <c r="N24" t="n">
+        <v>50</v>
+      </c>
+      <c r="O24" t="n">
+        <v>50</v>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Bitcoin</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" t="n">
-        <v>50</v>
-      </c>
-      <c r="E26" t="n">
-        <v>100</v>
-      </c>
-      <c r="F26" t="n">
-        <v>150</v>
-      </c>
-      <c r="G26" t="n">
-        <v>200</v>
-      </c>
-      <c r="H26" t="n">
-        <v>250</v>
-      </c>
-      <c r="I26" t="n">
-        <v>300</v>
-      </c>
-      <c r="J26" t="n">
-        <v>350</v>
-      </c>
-      <c r="K26" t="n">
-        <v>400</v>
-      </c>
-      <c r="L26" t="n">
-        <v>450</v>
-      </c>
-      <c r="M26" t="n">
-        <v>500</v>
-      </c>
-      <c r="N26" t="n">
-        <v>550</v>
-      </c>
-      <c r="O26" t="n">
-        <v>600</v>
-      </c>
-    </row>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.1667</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.1429</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.09089999999999999</v>
+      </c>
+    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ethereum</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
           <t>Crypto</t>
         </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" t="n">
-        <v>15</v>
-      </c>
-      <c r="E27" t="n">
-        <v>30</v>
-      </c>
-      <c r="F27" t="n">
-        <v>45</v>
-      </c>
-      <c r="G27" t="n">
-        <v>60</v>
-      </c>
-      <c r="H27" t="n">
-        <v>75</v>
-      </c>
-      <c r="I27" t="n">
-        <v>90</v>
-      </c>
-      <c r="J27" t="n">
-        <v>105</v>
-      </c>
-      <c r="K27" t="n">
-        <v>120</v>
-      </c>
-      <c r="L27" t="n">
-        <v>135</v>
-      </c>
-      <c r="M27" t="n">
-        <v>150</v>
-      </c>
-      <c r="N27" t="n">
-        <v>165</v>
-      </c>
-      <c r="O27" t="n">
-        <v>180</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Bitcoin</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E28" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="F28" t="n">
-        <v>195</v>
+        <v>150</v>
       </c>
       <c r="G28" t="n">
-        <v>260</v>
+        <v>200</v>
       </c>
       <c r="H28" t="n">
-        <v>325</v>
+        <v>250</v>
       </c>
       <c r="I28" t="n">
-        <v>390</v>
+        <v>300</v>
       </c>
       <c r="J28" t="n">
-        <v>455</v>
+        <v>350</v>
       </c>
       <c r="K28" t="n">
-        <v>520</v>
+        <v>400</v>
       </c>
       <c r="L28" t="n">
-        <v>585</v>
+        <v>450</v>
       </c>
       <c r="M28" t="n">
-        <v>650</v>
+        <v>500</v>
       </c>
       <c r="N28" t="n">
-        <v>715</v>
+        <v>550</v>
       </c>
       <c r="O28" t="n">
-        <v>780</v>
+        <v>600</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Gain/Loss</t>
-        </is>
+          <t>Ethereum</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Crypto</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>65</v>
+        <v>15</v>
       </c>
       <c r="E29" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="F29" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="G29" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H29" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="I29" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="J29" t="n">
-        <v>65</v>
+        <v>105</v>
       </c>
       <c r="K29" t="n">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="L29" t="n">
-        <v>65</v>
+        <v>135</v>
       </c>
       <c r="M29" t="n">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="N29" t="n">
-        <v>65</v>
+        <v>165</v>
       </c>
       <c r="O29" t="n">
-        <v>65</v>
+        <v>180</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>65</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>130</v>
       </c>
       <c r="F30" t="n">
-        <v>0.5</v>
+        <v>195</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3333</v>
+        <v>260</v>
       </c>
       <c r="H30" t="n">
-        <v>0.25</v>
+        <v>325</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2</v>
+        <v>390</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1667</v>
+        <v>455</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1429</v>
+        <v>520</v>
       </c>
       <c r="L30" t="n">
-        <v>0.125</v>
+        <v>585</v>
       </c>
       <c r="M30" t="n">
-        <v>0.1111</v>
+        <v>650</v>
       </c>
       <c r="N30" t="n">
-        <v>0.1</v>
+        <v>715</v>
       </c>
       <c r="O30" t="n">
-        <v>0.09089999999999999</v>
-      </c>
-    </row>
-    <row r="31"/>
+        <v>780</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Gain/Loss</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>65</v>
+      </c>
+      <c r="E31" t="n">
+        <v>65</v>
+      </c>
+      <c r="F31" t="n">
+        <v>65</v>
+      </c>
+      <c r="G31" t="n">
+        <v>65</v>
+      </c>
+      <c r="H31" t="n">
+        <v>65</v>
+      </c>
+      <c r="I31" t="n">
+        <v>65</v>
+      </c>
+      <c r="J31" t="n">
+        <v>65</v>
+      </c>
+      <c r="K31" t="n">
+        <v>65</v>
+      </c>
+      <c r="L31" t="n">
+        <v>65</v>
+      </c>
+      <c r="M31" t="n">
+        <v>65</v>
+      </c>
+      <c r="N31" t="n">
+        <v>65</v>
+      </c>
+      <c r="O31" t="n">
+        <v>65</v>
+      </c>
+    </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>WORK</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>TFR Lordo</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>4000</v>
-      </c>
-      <c r="D33" t="n">
-        <v>4250</v>
-      </c>
-      <c r="E33" t="n">
-        <v>4500</v>
-      </c>
-      <c r="F33" t="n">
-        <v>4750</v>
-      </c>
-      <c r="G33" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H33" t="n">
-        <v>5250</v>
-      </c>
-      <c r="I33" t="n">
-        <v>5500</v>
-      </c>
-      <c r="J33" t="n">
-        <v>5750</v>
-      </c>
-      <c r="K33" t="n">
-        <v>6000</v>
-      </c>
-      <c r="L33" t="n">
-        <v>6250</v>
-      </c>
-      <c r="M33" t="n">
-        <v>6500</v>
-      </c>
-      <c r="N33" t="n">
-        <v>6750</v>
-      </c>
-      <c r="O33" t="n">
-        <v>7000</v>
-      </c>
-    </row>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.1667</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.1429</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.1111</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.09089999999999999</v>
+      </c>
+    </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TFR Netto</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>3300</v>
-      </c>
-      <c r="D34" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3700</v>
-      </c>
-      <c r="F34" t="n">
-        <v>3900</v>
-      </c>
-      <c r="G34" t="n">
-        <v>4100</v>
-      </c>
-      <c r="H34" t="n">
-        <v>4300</v>
-      </c>
-      <c r="I34" t="n">
-        <v>4500</v>
-      </c>
-      <c r="J34" t="n">
-        <v>4700</v>
-      </c>
-      <c r="K34" t="n">
-        <v>4900</v>
-      </c>
-      <c r="L34" t="n">
-        <v>5100</v>
-      </c>
-      <c r="M34" t="n">
-        <v>5300</v>
-      </c>
-      <c r="N34" t="n">
-        <v>5500</v>
-      </c>
-      <c r="O34" t="n">
-        <v>5700</v>
+          <t>WORK</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>TFR Lordo</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7300</v>
+        <v>4000</v>
       </c>
       <c r="D35" t="n">
-        <v>7750</v>
+        <v>4250</v>
       </c>
       <c r="E35" t="n">
-        <v>8200</v>
+        <v>4500</v>
       </c>
       <c r="F35" t="n">
-        <v>8650</v>
+        <v>4750</v>
       </c>
       <c r="G35" t="n">
-        <v>9100</v>
+        <v>5000</v>
       </c>
       <c r="H35" t="n">
-        <v>9550</v>
+        <v>5250</v>
       </c>
       <c r="I35" t="n">
-        <v>10000</v>
+        <v>5500</v>
       </c>
       <c r="J35" t="n">
-        <v>10450</v>
+        <v>5750</v>
       </c>
       <c r="K35" t="n">
-        <v>10900</v>
+        <v>6000</v>
       </c>
       <c r="L35" t="n">
-        <v>11350</v>
+        <v>6250</v>
       </c>
       <c r="M35" t="n">
-        <v>11800</v>
+        <v>6500</v>
       </c>
       <c r="N35" t="n">
-        <v>12250</v>
+        <v>6750</v>
       </c>
       <c r="O35" t="n">
-        <v>12700</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Gain/Loss</t>
-        </is>
+          <t>TFR Netto</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3300</v>
       </c>
       <c r="D36" t="n">
-        <v>450</v>
+        <v>3500</v>
       </c>
       <c r="E36" t="n">
-        <v>450</v>
+        <v>3700</v>
       </c>
       <c r="F36" t="n">
-        <v>450</v>
+        <v>3900</v>
       </c>
       <c r="G36" t="n">
-        <v>450</v>
+        <v>4100</v>
       </c>
       <c r="H36" t="n">
-        <v>450</v>
+        <v>4300</v>
       </c>
       <c r="I36" t="n">
-        <v>450</v>
+        <v>4500</v>
       </c>
       <c r="J36" t="n">
-        <v>450</v>
+        <v>4700</v>
       </c>
       <c r="K36" t="n">
-        <v>450</v>
+        <v>4900</v>
       </c>
       <c r="L36" t="n">
-        <v>450</v>
+        <v>5100</v>
       </c>
       <c r="M36" t="n">
-        <v>450</v>
+        <v>5300</v>
       </c>
       <c r="N36" t="n">
-        <v>450</v>
+        <v>5500</v>
       </c>
       <c r="O36" t="n">
-        <v>450</v>
+        <v>5700</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>7300</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0616</v>
+        <v>7750</v>
       </c>
       <c r="E37" t="n">
-        <v>0.0581</v>
+        <v>8200</v>
       </c>
       <c r="F37" t="n">
-        <v>0.0549</v>
+        <v>8650</v>
       </c>
       <c r="G37" t="n">
-        <v>0.052</v>
+        <v>9100</v>
       </c>
       <c r="H37" t="n">
-        <v>0.0495</v>
+        <v>9550</v>
       </c>
       <c r="I37" t="n">
-        <v>0.0471</v>
+        <v>10000</v>
       </c>
       <c r="J37" t="n">
-        <v>0.045</v>
+        <v>10450</v>
       </c>
       <c r="K37" t="n">
-        <v>0.0431</v>
+        <v>10900</v>
       </c>
       <c r="L37" t="n">
-        <v>0.0413</v>
+        <v>11350</v>
       </c>
       <c r="M37" t="n">
-        <v>0.0396</v>
+        <v>11800</v>
       </c>
       <c r="N37" t="n">
-        <v>0.0381</v>
+        <v>12250</v>
       </c>
       <c r="O37" t="n">
-        <v>0.0367</v>
-      </c>
-    </row>
-    <row r="38"/>
+        <v>12700</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Gain/Loss</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>450</v>
+      </c>
+      <c r="E38" t="n">
+        <v>450</v>
+      </c>
+      <c r="F38" t="n">
+        <v>450</v>
+      </c>
+      <c r="G38" t="n">
+        <v>450</v>
+      </c>
+      <c r="H38" t="n">
+        <v>450</v>
+      </c>
+      <c r="I38" t="n">
+        <v>450</v>
+      </c>
+      <c r="J38" t="n">
+        <v>450</v>
+      </c>
+      <c r="K38" t="n">
+        <v>450</v>
+      </c>
+      <c r="L38" t="n">
+        <v>450</v>
+      </c>
+      <c r="M38" t="n">
+        <v>450</v>
+      </c>
+      <c r="N38" t="n">
+        <v>450</v>
+      </c>
+      <c r="O38" t="n">
+        <v>450</v>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Asset Allocation</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0616</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.0581</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.0549</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.0471</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.0431</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.0413</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.0396</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.0381</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.0367</v>
+      </c>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ETF</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>0.5</v>
+          <t>Asset Allocation</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ETF</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>Crypto</t>
         </is>
       </c>
-      <c r="C42" t="n">
+      <c r="C44" t="n">
         <v>0.2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Analisi Finanziarie: Entrate e uscite come un bilancio (macro categoria = somma delle voci)
- In alto i numeri dell'anno, una scheda colorata per macro categoria, grafico mese per
  mese per categoria, tabella con la riga della macro (somma) e sotto le sue voci
- Macro senza voci (ALTRO) su una riga; note a richiesta; voci a zero (13ESIMA) visibili
- L'import crea anche le voci ancora a zero e usa i nomi del file per le categorie già presenti
- Un colore diverso per ogni macro categoria; testo leggibile sui pulsanti nel tema scuro

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EU8iXu877ZDR8ixrLFK5MP
</commit_message>
<xml_diff>
--- a/finanza-personale/test/fixtures/file-completo-esempio.xlsx
+++ b/finanza-personale/test/fixtures/file-completo-esempio.xlsx
@@ -3916,7 +3916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4020,40 +4020,40 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="E3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="F3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="G3" t="n">
-        <v>1850</v>
+        <v>2510</v>
       </c>
       <c r="H3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="I3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="J3" t="n">
-        <v>1850</v>
+        <v>3860</v>
       </c>
       <c r="K3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="L3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="M3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="P3" t="n">
-        <v>18500</v>
+        <v>22450</v>
       </c>
       <c r="Q3" t="n">
-        <v>1850</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="4">
@@ -4100,266 +4100,435 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MUSICA</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>200</v>
-      </c>
-      <c r="E5" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>470.4</v>
-      </c>
-      <c r="H5" t="n">
-        <v>230</v>
-      </c>
-      <c r="I5" t="n">
-        <v>400</v>
-      </c>
-      <c r="J5" t="n">
-        <v>600</v>
-      </c>
-      <c r="K5" t="n">
-        <v>332.25</v>
-      </c>
-      <c r="L5" t="n">
-        <v>98.09999999999999</v>
-      </c>
-      <c r="M5" t="n">
-        <v>250</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>13ESIMA</t>
+        </is>
       </c>
       <c r="P5" t="n">
-        <v>2626.25</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>262.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>DJ</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Serate</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>200</v>
-      </c>
-      <c r="F6" t="n">
-        <v>350</v>
-      </c>
-      <c r="H6" t="n">
-        <v>150</v>
-      </c>
-      <c r="I6" t="n">
-        <v>400</v>
+          <t>14ESIMA</t>
+        </is>
       </c>
       <c r="J6" t="n">
-        <v>600</v>
-      </c>
-      <c r="K6" t="n">
-        <v>300</v>
-      </c>
-      <c r="M6" t="n">
-        <v>250</v>
+        <v>1850</v>
       </c>
       <c r="P6" t="n">
-        <v>2250</v>
+        <v>1850</v>
       </c>
       <c r="Q6" t="n">
-        <v>225</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>PRODUZIONE</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Groover</t>
-        </is>
+          <t>BUONI PASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>160</v>
       </c>
       <c r="E7" t="n">
-        <v>45.5</v>
+        <v>160</v>
+      </c>
+      <c r="F7" t="n">
+        <v>160</v>
+      </c>
+      <c r="G7" t="n">
+        <v>160</v>
       </c>
       <c r="H7" t="n">
-        <v>80</v>
+        <v>160</v>
+      </c>
+      <c r="I7" t="n">
+        <v>160</v>
+      </c>
+      <c r="J7" t="n">
+        <v>160</v>
       </c>
       <c r="K7" t="n">
-        <v>32.25</v>
+        <v>160</v>
+      </c>
+      <c r="L7" t="n">
+        <v>160</v>
+      </c>
+      <c r="M7" t="n">
+        <v>160</v>
       </c>
       <c r="P7" t="n">
-        <v>157.75</v>
+        <v>1600</v>
       </c>
       <c r="Q7" t="n">
-        <v>15.78</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>SIAE</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>120.4</v>
-      </c>
-      <c r="L8" t="n">
-        <v>98.09999999999999</v>
+          <t>WELFARE</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>500</v>
       </c>
       <c r="P8" t="n">
-        <v>218.5</v>
+        <v>500</v>
       </c>
       <c r="Q8" t="n">
-        <v>21.85</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INT. BANCA</t>
+          <t>MUSICA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>12.1</v>
+        <v>200</v>
       </c>
       <c r="E9" t="n">
-        <v>11.8</v>
+        <v>95.5</v>
       </c>
       <c r="F9" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="G9" t="n">
-        <v>12</v>
+        <v>470.4</v>
       </c>
       <c r="H9" t="n">
-        <v>12.2</v>
+        <v>230</v>
       </c>
       <c r="I9" t="n">
-        <v>11.9</v>
+        <v>430</v>
       </c>
       <c r="J9" t="n">
-        <v>12.3</v>
+        <v>600</v>
       </c>
       <c r="K9" t="n">
-        <v>12.5</v>
+        <v>332.25</v>
       </c>
       <c r="L9" t="n">
-        <v>12</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>12.6</v>
+        <v>250</v>
       </c>
       <c r="P9" t="n">
-        <v>121.8</v>
+        <v>2706.25</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.18</v>
+        <v>270.62</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>INTERESSI</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+          <t>ALTRO</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I10" t="n">
+        <v>30</v>
+      </c>
+      <c r="P10" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DJ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Serate</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" t="n">
+        <v>350</v>
+      </c>
+      <c r="H11" t="n">
+        <v>150</v>
+      </c>
+      <c r="I11" t="n">
+        <v>400</v>
+      </c>
+      <c r="J11" t="n">
+        <v>600</v>
+      </c>
+      <c r="K11" t="n">
+        <v>300</v>
+      </c>
+      <c r="M11" t="n">
+        <v>250</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2250</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PRODUZIONE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Groover</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>80</v>
+      </c>
+      <c r="K12" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="P12" t="n">
+        <v>157.75</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>15.78</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GRAFICHE</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>120.4</v>
+      </c>
+      <c r="L13" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="P13" t="n">
+        <v>218.5</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>21.85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>INT. BANCA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>14</v>
+      </c>
+      <c r="H14" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="J14" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="K14" t="n">
+        <v>15</v>
+      </c>
+      <c r="L14" t="n">
+        <v>14</v>
+      </c>
+      <c r="M14" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="P14" t="n">
+        <v>143.6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>14.36</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>Conto deposito</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D16" t="n">
         <v>12.1</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E16" t="n">
         <v>11.8</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F16" t="n">
         <v>12.4</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G16" t="n">
         <v>12</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H16" t="n">
         <v>12.2</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I16" t="n">
         <v>11.9</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J16" t="n">
         <v>12.3</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K16" t="n">
         <v>12.5</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L16" t="n">
         <v>12</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M16" t="n">
         <v>12.6</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P16" t="n">
         <v>121.8</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q16" t="n">
         <v>12.18</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ALTRO</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>75</v>
+      </c>
+      <c r="K17" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>2062.1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1907.3</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2332.8</v>
-      </c>
-      <c r="G12" t="n">
-        <v>1862</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2092.2</v>
-      </c>
-      <c r="I12" t="n">
-        <v>2261.9</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2462.3</v>
-      </c>
-      <c r="K12" t="n">
-        <v>2194.75</v>
-      </c>
-      <c r="L12" t="n">
-        <v>1960.1</v>
-      </c>
-      <c r="M12" t="n">
-        <v>2112.6</v>
-      </c>
-      <c r="N12" t="n">
+      <c r="D19" t="n">
+        <v>2224.2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2119.1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2570.2</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2524</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2254.4</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2453.8</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4474.6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>2377.25</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2122.1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2275.2</v>
+      </c>
+      <c r="N19" t="n">
         <v>0</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O19" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="n">
-        <v>21248.05</v>
+      <c r="P19" t="n">
+        <v>25394.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Analisi Finanziarie: Entrate e uscite come un bilancio (macro categoria = somma delle voci) (#92)
- In alto i numeri dell'anno, una scheda colorata per macro categoria, grafico mese per
  mese per categoria, tabella con la riga della macro (somma) e sotto le sue voci
- Macro senza voci (ALTRO) su una riga; note a richiesta; voci a zero (13ESIMA) visibili
- L'import crea anche le voci ancora a zero e usa i nomi del file per le categorie già presenti
- Un colore diverso per ogni macro categoria; testo leggibile sui pulsanti nel tema scuro


Claude-Session: https://claude.ai/code/session_01EU8iXu877ZDR8ixrLFK5MP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finanza-personale/test/fixtures/file-completo-esempio.xlsx
+++ b/finanza-personale/test/fixtures/file-completo-esempio.xlsx
@@ -3916,7 +3916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4020,40 +4020,40 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="E3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="F3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="G3" t="n">
-        <v>1850</v>
+        <v>2510</v>
       </c>
       <c r="H3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="I3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="J3" t="n">
-        <v>1850</v>
+        <v>3860</v>
       </c>
       <c r="K3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="L3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="M3" t="n">
-        <v>1850</v>
+        <v>2010</v>
       </c>
       <c r="P3" t="n">
-        <v>18500</v>
+        <v>22450</v>
       </c>
       <c r="Q3" t="n">
-        <v>1850</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="4">
@@ -4100,266 +4100,435 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MUSICA</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>200</v>
-      </c>
-      <c r="E5" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>470.4</v>
-      </c>
-      <c r="H5" t="n">
-        <v>230</v>
-      </c>
-      <c r="I5" t="n">
-        <v>400</v>
-      </c>
-      <c r="J5" t="n">
-        <v>600</v>
-      </c>
-      <c r="K5" t="n">
-        <v>332.25</v>
-      </c>
-      <c r="L5" t="n">
-        <v>98.09999999999999</v>
-      </c>
-      <c r="M5" t="n">
-        <v>250</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>13ESIMA</t>
+        </is>
       </c>
       <c r="P5" t="n">
-        <v>2626.25</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>262.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>DJ</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Serate</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>200</v>
-      </c>
-      <c r="F6" t="n">
-        <v>350</v>
-      </c>
-      <c r="H6" t="n">
-        <v>150</v>
-      </c>
-      <c r="I6" t="n">
-        <v>400</v>
+          <t>14ESIMA</t>
+        </is>
       </c>
       <c r="J6" t="n">
-        <v>600</v>
-      </c>
-      <c r="K6" t="n">
-        <v>300</v>
-      </c>
-      <c r="M6" t="n">
-        <v>250</v>
+        <v>1850</v>
       </c>
       <c r="P6" t="n">
-        <v>2250</v>
+        <v>1850</v>
       </c>
       <c r="Q6" t="n">
-        <v>225</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>PRODUZIONE</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Groover</t>
-        </is>
+          <t>BUONI PASTO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>160</v>
       </c>
       <c r="E7" t="n">
-        <v>45.5</v>
+        <v>160</v>
+      </c>
+      <c r="F7" t="n">
+        <v>160</v>
+      </c>
+      <c r="G7" t="n">
+        <v>160</v>
       </c>
       <c r="H7" t="n">
-        <v>80</v>
+        <v>160</v>
+      </c>
+      <c r="I7" t="n">
+        <v>160</v>
+      </c>
+      <c r="J7" t="n">
+        <v>160</v>
       </c>
       <c r="K7" t="n">
-        <v>32.25</v>
+        <v>160</v>
+      </c>
+      <c r="L7" t="n">
+        <v>160</v>
+      </c>
+      <c r="M7" t="n">
+        <v>160</v>
       </c>
       <c r="P7" t="n">
-        <v>157.75</v>
+        <v>1600</v>
       </c>
       <c r="Q7" t="n">
-        <v>15.78</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>SIAE</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>120.4</v>
-      </c>
-      <c r="L8" t="n">
-        <v>98.09999999999999</v>
+          <t>WELFARE</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>500</v>
       </c>
       <c r="P8" t="n">
-        <v>218.5</v>
+        <v>500</v>
       </c>
       <c r="Q8" t="n">
-        <v>21.85</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INT. BANCA</t>
+          <t>MUSICA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>12.1</v>
+        <v>200</v>
       </c>
       <c r="E9" t="n">
-        <v>11.8</v>
+        <v>95.5</v>
       </c>
       <c r="F9" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="G9" t="n">
-        <v>12</v>
+        <v>470.4</v>
       </c>
       <c r="H9" t="n">
-        <v>12.2</v>
+        <v>230</v>
       </c>
       <c r="I9" t="n">
-        <v>11.9</v>
+        <v>430</v>
       </c>
       <c r="J9" t="n">
-        <v>12.3</v>
+        <v>600</v>
       </c>
       <c r="K9" t="n">
-        <v>12.5</v>
+        <v>332.25</v>
       </c>
       <c r="L9" t="n">
-        <v>12</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>12.6</v>
+        <v>250</v>
       </c>
       <c r="P9" t="n">
-        <v>121.8</v>
+        <v>2706.25</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.18</v>
+        <v>270.62</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>INTERESSI</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+          <t>ALTRO</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>50</v>
+      </c>
+      <c r="I10" t="n">
+        <v>30</v>
+      </c>
+      <c r="P10" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DJ</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Serate</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" t="n">
+        <v>350</v>
+      </c>
+      <c r="H11" t="n">
+        <v>150</v>
+      </c>
+      <c r="I11" t="n">
+        <v>400</v>
+      </c>
+      <c r="J11" t="n">
+        <v>600</v>
+      </c>
+      <c r="K11" t="n">
+        <v>300</v>
+      </c>
+      <c r="M11" t="n">
+        <v>250</v>
+      </c>
+      <c r="P11" t="n">
+        <v>2250</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PRODUZIONE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Groover</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>80</v>
+      </c>
+      <c r="K12" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="P12" t="n">
+        <v>157.75</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>15.78</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GRAFICHE</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>120.4</v>
+      </c>
+      <c r="L13" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="P13" t="n">
+        <v>218.5</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>21.85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>INT. BANCA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>14</v>
+      </c>
+      <c r="H14" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="J14" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="K14" t="n">
+        <v>15</v>
+      </c>
+      <c r="L14" t="n">
+        <v>14</v>
+      </c>
+      <c r="M14" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="P14" t="n">
+        <v>143.6</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>14.36</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K15" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P15" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>Conto deposito</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D16" t="n">
         <v>12.1</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E16" t="n">
         <v>11.8</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F16" t="n">
         <v>12.4</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G16" t="n">
         <v>12</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H16" t="n">
         <v>12.2</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I16" t="n">
         <v>11.9</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J16" t="n">
         <v>12.3</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K16" t="n">
         <v>12.5</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L16" t="n">
         <v>12</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M16" t="n">
         <v>12.6</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P16" t="n">
         <v>121.8</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q16" t="n">
         <v>12.18</v>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ALTRO</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>75</v>
+      </c>
+      <c r="K17" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>2062.1</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1907.3</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2332.8</v>
-      </c>
-      <c r="G12" t="n">
-        <v>1862</v>
-      </c>
-      <c r="H12" t="n">
-        <v>2092.2</v>
-      </c>
-      <c r="I12" t="n">
-        <v>2261.9</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2462.3</v>
-      </c>
-      <c r="K12" t="n">
-        <v>2194.75</v>
-      </c>
-      <c r="L12" t="n">
-        <v>1960.1</v>
-      </c>
-      <c r="M12" t="n">
-        <v>2112.6</v>
-      </c>
-      <c r="N12" t="n">
+      <c r="D19" t="n">
+        <v>2224.2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2119.1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2570.2</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2524</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2254.4</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2453.8</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4474.6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>2377.25</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2122.1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2275.2</v>
+      </c>
+      <c r="N19" t="n">
         <v>0</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O19" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="n">
-        <v>21248.05</v>
+      <c r="P19" t="n">
+        <v>25394.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Analisi Finanziarie: statistiche fuori dalle entrate, impostazioni con il menu delle sezioni
- Le righe di riepilogo del foglio (Liquidità a fine 2025, tutto sotto la riga TOTALE) non
  sono entrate: si saltano nell'import e si tolgono se già importate
- Impostazioni: menu delle sezioni a sinistra e sezioni una sotto l'altra; Categorie come
  riepilogo per macro categoria

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EU8iXu877ZDR8ixrLFK5MP
</commit_message>
<xml_diff>
--- a/finanza-personale/test/fixtures/file-completo-esempio.xlsx
+++ b/finanza-personale/test/fixtures/file-completo-esempio.xlsx
@@ -3916,7 +3916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4016,519 +4016,540 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>LIQUIDITÀ A FINE 2025</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15230.45</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>LAVORO</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>2010</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>2010</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F4" t="n">
         <v>2010</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G4" t="n">
         <v>2510</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H4" t="n">
         <v>2010</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I4" t="n">
         <v>2010</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J4" t="n">
         <v>3860</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K4" t="n">
         <v>2010</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L4" t="n">
         <v>2010</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M4" t="n">
         <v>2010</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P4" t="n">
         <v>22450</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q4" t="n">
         <v>2245</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>STIPENDIO</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="M4" t="n">
-        <v>1850</v>
-      </c>
-      <c r="P4" t="n">
-        <v>18500</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>1850</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>13ESIMA</t>
-        </is>
+          <t>STIPENDIO</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1850</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1850</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>18500</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>14ESIMA</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>1850</v>
+          <t>13ESIMA</t>
+        </is>
       </c>
       <c r="P6" t="n">
-        <v>1850</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>185</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>BUONI PASTO</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>160</v>
-      </c>
-      <c r="E7" t="n">
-        <v>160</v>
-      </c>
-      <c r="F7" t="n">
-        <v>160</v>
-      </c>
-      <c r="G7" t="n">
-        <v>160</v>
-      </c>
-      <c r="H7" t="n">
-        <v>160</v>
-      </c>
-      <c r="I7" t="n">
-        <v>160</v>
+          <t>14ESIMA</t>
+        </is>
       </c>
       <c r="J7" t="n">
-        <v>160</v>
-      </c>
-      <c r="K7" t="n">
-        <v>160</v>
-      </c>
-      <c r="L7" t="n">
-        <v>160</v>
-      </c>
-      <c r="M7" t="n">
-        <v>160</v>
+        <v>1850</v>
       </c>
       <c r="P7" t="n">
-        <v>1600</v>
+        <v>1850</v>
       </c>
       <c r="Q7" t="n">
-        <v>160</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
+          <t>BUONI PASTO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>160</v>
+      </c>
+      <c r="E8" t="n">
+        <v>160</v>
+      </c>
+      <c r="F8" t="n">
+        <v>160</v>
+      </c>
+      <c r="G8" t="n">
+        <v>160</v>
+      </c>
+      <c r="H8" t="n">
+        <v>160</v>
+      </c>
+      <c r="I8" t="n">
+        <v>160</v>
+      </c>
+      <c r="J8" t="n">
+        <v>160</v>
+      </c>
+      <c r="K8" t="n">
+        <v>160</v>
+      </c>
+      <c r="L8" t="n">
+        <v>160</v>
+      </c>
+      <c r="M8" t="n">
+        <v>160</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1600</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
           <t>WELFARE</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="G9" t="n">
         <v>500</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P9" t="n">
         <v>500</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q9" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>MUSICA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>200</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E10" t="n">
         <v>95.5</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F10" t="n">
         <v>470.4</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H10" t="n">
         <v>230</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I10" t="n">
         <v>430</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J10" t="n">
         <v>600</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K10" t="n">
         <v>332.25</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L10" t="n">
         <v>98.09999999999999</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M10" t="n">
         <v>250</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P10" t="n">
         <v>2706.25</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q10" t="n">
         <v>270.62</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ALTRO</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>50</v>
-      </c>
-      <c r="I10" t="n">
-        <v>30</v>
-      </c>
-      <c r="P10" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>DJ</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Serate</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>200</v>
-      </c>
-      <c r="F11" t="n">
-        <v>350</v>
-      </c>
-      <c r="H11" t="n">
-        <v>150</v>
+          <t>ALTRO</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>50</v>
       </c>
       <c r="I11" t="n">
-        <v>400</v>
-      </c>
-      <c r="J11" t="n">
-        <v>600</v>
-      </c>
-      <c r="K11" t="n">
-        <v>300</v>
-      </c>
-      <c r="M11" t="n">
-        <v>250</v>
+        <v>30</v>
       </c>
       <c r="P11" t="n">
-        <v>2250</v>
+        <v>80</v>
       </c>
       <c r="Q11" t="n">
-        <v>225</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>PRODUZIONE</t>
+          <t>DJ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Groover</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>45.5</v>
+          <t>Serate</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>200</v>
+      </c>
+      <c r="F12" t="n">
+        <v>350</v>
       </c>
       <c r="H12" t="n">
-        <v>80</v>
+        <v>150</v>
+      </c>
+      <c r="I12" t="n">
+        <v>400</v>
+      </c>
+      <c r="J12" t="n">
+        <v>600</v>
       </c>
       <c r="K12" t="n">
-        <v>32.25</v>
+        <v>300</v>
+      </c>
+      <c r="M12" t="n">
+        <v>250</v>
       </c>
       <c r="P12" t="n">
-        <v>157.75</v>
+        <v>2250</v>
       </c>
       <c r="Q12" t="n">
-        <v>15.78</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
+          <t>PRODUZIONE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Groover</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>80</v>
+      </c>
+      <c r="K13" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="P13" t="n">
+        <v>157.75</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>15.78</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
           <t>GRAFICHE</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F14" t="n">
         <v>120.4</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L14" t="n">
         <v>98.09999999999999</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P14" t="n">
         <v>218.5</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q14" t="n">
         <v>21.85</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>INT. BANCA</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>14.2</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E15" t="n">
         <v>13.6</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F15" t="n">
         <v>14.8</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G15" t="n">
         <v>14</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H15" t="n">
         <v>14.4</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I15" t="n">
         <v>13.8</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J15" t="n">
         <v>14.6</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K15" t="n">
         <v>15</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L15" t="n">
         <v>14</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M15" t="n">
         <v>15.2</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P15" t="n">
         <v>143.6</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q15" t="n">
         <v>14.36</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F15" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="G15" t="n">
-        <v>2</v>
-      </c>
-      <c r="H15" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="J15" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="K15" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L15" t="n">
-        <v>2</v>
-      </c>
-      <c r="M15" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="P15" t="n">
-        <v>21.8</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>2.18</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J16" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P16" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
           <t>CD</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Conto deposito</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>12.1</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E17" t="n">
         <v>11.8</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F17" t="n">
         <v>12.4</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G17" t="n">
         <v>12</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H17" t="n">
         <v>12.2</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I17" t="n">
         <v>11.9</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J17" t="n">
         <v>12.3</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K17" t="n">
         <v>12.5</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L17" t="n">
         <v>12</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M17" t="n">
         <v>12.6</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>121.8</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>12.18</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>ALTRO</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>75</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>20</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>95</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>9.5</v>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D20" t="n">
         <v>2224.2</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E20" t="n">
         <v>2119.1</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F20" t="n">
         <v>2570.2</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G20" t="n">
         <v>2524</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H20" t="n">
         <v>2254.4</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I20" t="n">
         <v>2453.8</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J20" t="n">
         <v>4474.6</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K20" t="n">
         <v>2377.25</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L20" t="n">
         <v>2122.1</v>
       </c>
-      <c r="M19" t="n">
+      <c r="M20" t="n">
         <v>2275.2</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N20" t="n">
         <v>0</v>
       </c>
-      <c r="O19" t="n">
+      <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="P19" t="n">
+      <c r="P20" t="n">
         <v>25394.85</v>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RISPARMIO MEDIO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>812.5</v>
       </c>
     </row>
   </sheetData>
@@ -4542,7 +4563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4828,6 +4849,17 @@
       </c>
       <c r="P7" t="n">
         <v>10283</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RISPARMIO MEDIO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>812.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>